<commit_message>
feat(contratos): Excel de pendências com rateio por NF (cabeçalho + itens)
- processarPlanilhaContratos: colunas passam a ser Tipo | Contrato |
  Projeto | Valor | Data | Nº da NF | Observações (sem "Fornecedor/
  Terceiro" — vem do contrato). PAGAMENTO: linhas com o mesmo
  Contrato + Nº da NF viram 1 pendência (cabeçalho, valor = Σ) com N
  itens de rateio em contratos_pendencias_itens; sem Nº da NF, 1 linha =
  1 pendência de 1 projeto. PROPOSTA continua 1 linha = 1 pendência.
- Relatório de import conta pendências criadas.
- index.html: descrição das colunas atualizada.
- docs/exemplo_pendencias_contratos.xlsx: regerado (linhas 2+3 = 1 NF
  rateada, + casos de erro/ERRO_LEITURA).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/exemplo_pendencias_contratos.xlsx
+++ b/docs/exemplo_pendencias_contratos.xlsx
@@ -426,17 +426,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="26" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="44" customWidth="1" min="7" max="7"/>
-    <col width="24" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -457,27 +456,22 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Fornecedor/Terceiro</t>
+          <t>Valor</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Valor</t>
+          <t>Data de Referência</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Data de Referência</t>
+          <t>Nº da NF</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Observações</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Nome do Arquivo da NF</t>
         </is>
       </c>
     </row>
@@ -497,34 +491,29 @@
           <t>PRJ-FY27-002-TES</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>ACME Servicos Ltda</t>
-        </is>
-      </c>
-      <c r="E2" t="n">
-        <v>15000</v>
+      <c r="D2" t="n">
+        <v>9000</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>05/09/2026</t>
+        </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>05/09/2026</t>
+          <t>NF-1001</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Parcela 1/3 da execucao</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>nf-acme-001.pdf</t>
+          <t>Rateio NF 1001 - projeto TES</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Proposta</t>
+          <t>Pagamento</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -537,27 +526,22 @@
           <t>PRJ-FY27-003-RHU</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>ACME Servicos Ltda</t>
-        </is>
-      </c>
-      <c r="E3" t="n">
-        <v>42000</v>
+      <c r="D3" t="n">
+        <v>6000</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>05/09/2026</t>
+        </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>01/09/2026</t>
+          <t>NF-1001</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Proposta tecnica revisada</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>proposta-acme.pdf</t>
+          <t>Rateio NF 1001 - projeto RHU</t>
         </is>
       </c>
     </row>
@@ -577,30 +561,29 @@
           <t>PRJ-FY27-002-TES</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Beta Consultoria SA</t>
-        </is>
-      </c>
-      <c r="E4" t="n">
+      <c r="D4" t="n">
         <v>8000</v>
       </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>08/09/2026</t>
+        </is>
+      </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>08/09/2026</t>
+          <t>NF-2002</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Consultoria set/2026</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr"/>
+          <t>NF de 1 projeto so</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Reembolso</t>
+          <t>Proposta</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -610,33 +593,28 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>PRJ-FY27-002-TES</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>ACME Servicos Ltda</t>
-        </is>
-      </c>
-      <c r="E5" t="n">
-        <v>500</v>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>10/09/2026</t>
-        </is>
-      </c>
+          <t>PRJ-FY27-003-RHU</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>42000</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>01/09/2026</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
-          <t>linha invalida: tipo nao reconhecido</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr"/>
+          <t>Proposta tecnica</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Pagamento</t>
+          <t>Reembolso</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -649,23 +627,24 @@
           <t>PRJ-FY27-002-TES</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>ACME Servicos Ltda</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr"/>
+      <c r="D6" t="n">
+        <v>500</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>10/09/2026</t>
+        </is>
+      </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>10/09/2026</t>
+          <t>NF-9</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>linha invalida: valor em branco</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr"/>
+          <t>linha invalida: tipo</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -683,25 +662,22 @@
           <t>PRJ-FY27-002-TES</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>ACME Servicos Ltda</t>
-        </is>
-      </c>
-      <c r="E7" t="n">
-        <v>1000</v>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>10/09/2026</t>
+        </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>NF-8</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>linha invalida: data fora do formato dd/mm/aaaa</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr"/>
+          <t>linha invalida: sem valor</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -711,7 +687,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>CT-9999-INEXISTENTE</t>
+          <t>CT-9999-XX</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -719,61 +695,24 @@
           <t>PRJ-FY27-002-TES</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Gamma Tech</t>
-        </is>
-      </c>
-      <c r="E8" t="n">
+      <c r="D8" t="n">
         <v>3000</v>
       </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>12/09/2026</t>
+        </is>
+      </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>12/09/2026</t>
+          <t>NF-7</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>contrato nao localizado -&gt; pendencia ERRO_LEITURA</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Proposta</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>CT-2026-001</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>PROJETO-INEXISTENTE</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>ACME Servicos Ltda</t>
-        </is>
-      </c>
-      <c r="E9" t="n">
-        <v>2000</v>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>12/09/2026</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>projeto nao localizado -&gt; pendencia ERRO_LEITURA</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr"/>
+          <t>contrato inexistente -&gt; ERRO_LEITURA</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -786,16 +725,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A22"/>
+  <dimension ref="A1:A13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="110" customWidth="1" min="1" max="1"/>
+    <col width="95" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Arquivo de teste — Pendencias de Contratos (Fase A)</t>
+          <t>Arquivo de teste — Pendencias de Contratos (Release 1, rateio por NF)</t>
         </is>
       </c>
     </row>
@@ -805,132 +744,73 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>O sistema le a PRIMEIRA aba ('Lancamentos'). Cabecalho na linha 1, com estes rotulos exatos:</t>
+          <t>Aba lida: a primeira (Lancamentos).</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Tipo de Lancamento | Contrato | Projeto | Fornecedor/Terceiro | Valor | Data de Referencia | Observacoes | Nome do Arquivo da NF</t>
+          <t>PAGAMENTO: linhas 2 e 3 tem o MESMO Contrato (CT-2026-001) e Nº da NF (NF-1001)</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr"/>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   -&gt; viram 1 pendencia de R$ 15.000 com rateio: TES 9.000 + RHU 6.000.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Comportamento esperado ao subir este arquivo:</t>
+          <t>Linha 4 (CT-2026-002 / NF-2002): pendencia de pagamento de 1 projeto so.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Linhas 2 e 3 (Pagamento) e linha 3 (Proposta): viram pendencias PENDENTE se o Contrato e o Projeto</t>
+          <t>Linha 5 (Proposta): 1 pendencia de proposta (sem rateio).</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">      existirem na sua base. Senao, viram ERRO_LEITURA (a pendencia e criada; voce resolve contrato/projeto</t>
+          <t>Linha 6 (Reembolso): relatorio de erros (tipo invalido).</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">      no modal 'Detalhar').</t>
+          <t>Linha 7 (sem Valor): relatorio de erros.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Linha 5 ('Reembolso'): NAO vira pendencia — entra no relatorio de erros (tipo invalido).</t>
+          <t>Linha 8 (CT-9999-XX): pendencia ERRO_LEITURA (contrato nao localizado).</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Linha 6 (sem Valor): relatorio de erros.</t>
-        </is>
-      </c>
+      <c r="A11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Linha 7 (data '2026-09-15'): relatorio de erros (use dd/mm/aaaa).</t>
+          <t>Ajuste Contrato/Projeto para casar com o que voce cadastrou em Fornecedores /</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Linhas 8 e 9: pendencia criada como ERRO_LEITURA (contrato/projeto nao localizado).</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Para um teste 'feliz' completo:</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  1. Cadastre em 'Contratos Terceirizados' um contrato com numero CT-2026-001 (e CT-2026-002 se quiser).</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  2. Em 'Contratos por Projeto', vincule esse contrato a um projeto (o codigo que voce usar na coluna Projeto).</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  3. Ajuste as colunas Contrato/Projeto das linhas 2-4 para casar com o que voce cadastrou.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  4. Suba o arquivo. As linhas boas viram PENDENTE; anexe a NF (classificacao 'Nota Fiscal') e Aprovar.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">     Pagamento -&gt; grava em contratos_pagamentos; Proposta -&gt; grava em contratos_propostas.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  5. Teste tambem: aprovar sem NF (bloqueia) -&gt; 'Dispensar NF...' com justificativa -&gt; aprovar.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  6. Rejeitar uma pendencia com motivo.</t>
+          <t>Contratos Terceirizados / Vincular Projeto e Contrato.</t>
         </is>
       </c>
     </row>

</xml_diff>